<commit_message>
Add sort control; fix Spotify links to point at correct albums
Add a Date/Name sort toggle above the release list, defaulting to
newest-first, with click-to-flip direction.

Also fix five releases in credits.xlsx whose Spotify links pointed at
an individual track instead of the containing release (San Fermin's
"Arms" was linked to an unrelated same-titled 2023 song rather than
the actual album; four singles were linked to the bare track instead
of their single/EP page). Resolved via each track's own og:music:album
metadata rather than guessing from search results, since fuzzy name
search returned same-titled but unrelated recordings for several of
these.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/credits.xlsx
+++ b/data/credits.xlsx
@@ -399,17 +399,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I44"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="6.83203125" customWidth="1"/>
-    <col min="5" max="5" width="40.83203125" customWidth="1"/>
-    <col min="6" max="6" width="40.83203125" customWidth="1"/>
-    <col min="7" max="7" width="40.83203125" customWidth="1"/>
-    <col min="8" max="8" width="50.83203125" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -486,7 +475,7 @@
         <v>https://sanferminband.bandcamp.com/album/arms</v>
       </c>
       <c r="F3" t="str">
-        <v>https://open.spotify.com/track/4cQpA3lSvchIKnmo1fzEAL</v>
+        <v>https://open.spotify.com/album/5grHCZZ9MudkWc1yFq8RQC</v>
       </c>
       <c r="G3" t="str">
         <v/>
@@ -863,7 +852,7 @@
         <v/>
       </c>
       <c r="F16" t="str">
-        <v>https://open.spotify.com/track/67djP6VPqGDjG5jJgBEuQb</v>
+        <v>https://open.spotify.com/album/7weMOuQtaLZ5IM1FFpSv8v</v>
       </c>
       <c r="G16" t="str">
         <v/>
@@ -1124,7 +1113,7 @@
         <v/>
       </c>
       <c r="F25" t="str">
-        <v>https://open.spotify.com/track/45IryAtCyBE0zAdYe77Lll</v>
+        <v>https://open.spotify.com/album/5YCkSdO04tHwrurgYzN09v</v>
       </c>
       <c r="G25" t="str">
         <v/>
@@ -1211,7 +1200,7 @@
         <v/>
       </c>
       <c r="F28" t="str">
-        <v>https://open.spotify.com/track/0MBupnLliwp226j5RSaPt0</v>
+        <v>https://open.spotify.com/album/4DRVBIISdoxJAb7Syh3gSt</v>
       </c>
       <c r="G28" t="str">
         <v/>
@@ -1530,7 +1519,7 @@
         <v/>
       </c>
       <c r="F39" t="str">
-        <v>https://open.spotify.com/track/2um4ISitgBDdMSZaiPyaIb</v>
+        <v>https://open.spotify.com/album/4ek7xLvUQ1XJW5iVGjRg6l</v>
       </c>
       <c r="G39" t="str">
         <v/>
@@ -1697,12 +1686,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D268"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="32.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="50.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>